<commit_message>
Update text files (new languages)
</commit_message>
<xml_diff>
--- a/OpenSesame-local/mbrt_files/Block_messages.xlsx
+++ b/OpenSesame-local/mbrt_files/Block_messages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdabb12e9f34f4c5/10_Paper/105_MIA/10_BAS_Collab/MBRT/MBRT-OpenSesame-LL/MBRT_online/mbrt_files/xlsx-files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdabb12e9f34f4c5/10_Paper/105_MIA/10_BAS_Collab/MBRT/OpenSesame-local/mbrt_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="13_ncr:1_{C85E377C-CD68-4776-A203-A73B30935160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F0D0A27-8E63-4BA2-9591-62B9A71467E5}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{C85E377C-CD68-4776-A203-A73B30935160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C60D8B10-A3BA-42DD-B9ED-CA5D85335A91}"/>
   <bookViews>
-    <workbookView xWindow="44880" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{3128DB0A-6163-4D40-98DA-1667AB584357}"/>
+    <workbookView xWindow="37263" yWindow="774" windowWidth="26083" windowHeight="13830" xr2:uid="{3128DB0A-6163-4D40-98DA-1667AB584357}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>block_pause_msg_en</t>
   </si>
@@ -108,6 +109,78 @@
   </si>
   <si>
     <t>Es folgt nun der letzte Block.&lt;br&gt;&lt;br&gt;Erinnerung: Antworten Sie so &lt;b&gt;schnell und korrekt&lt;/b&gt; wie möglich.</t>
+  </si>
+  <si>
+    <t>Ha completado el primer bloque.</t>
+  </si>
+  <si>
+    <t>Vous avez terminé le premier bloc.</t>
+  </si>
+  <si>
+    <t>Ha completado el segundo bloque.</t>
+  </si>
+  <si>
+    <t>Vous avez terminé le deuxième bloc.</t>
+  </si>
+  <si>
+    <t>Ha completado el tercer bloque.</t>
+  </si>
+  <si>
+    <t>Vous avez terminé le troisième bloc.</t>
+  </si>
+  <si>
+    <t>Ha completado el último bloque.</t>
+  </si>
+  <si>
+    <t>Vous avez terminé le dernier bloc.</t>
+  </si>
+  <si>
+    <t>single_block_msg_es</t>
+  </si>
+  <si>
+    <t>block_msg_es</t>
+  </si>
+  <si>
+    <t>block_pause_msg_es</t>
+  </si>
+  <si>
+    <t>single_block_msg_fr</t>
+  </si>
+  <si>
+    <t>block_msg_fr</t>
+  </si>
+  <si>
+    <t>block_pause_msg_fr</t>
+  </si>
+  <si>
+    <t>Ahora completará un bloque de ensayos,&lt;br&gt;en los que mediremos sus datos.&lt;br&gt;&lt;b&gt;Cada ensayo cuenta.&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Ahora completará &lt;b&gt;4 bloques&lt;/b&gt; de ensayos,&lt;br&gt;en los que mediremos sus datos.&lt;br&gt;&lt;b&gt;Cada ensayo cuenta.&lt;/b&gt;&lt;br&gt;&lt;br&gt;Entre los bloques puede hacer una pausa.&lt;br&gt;&lt;br&gt;El primer bloque comienza al pulsar la tecla ESPACIO.</t>
+  </si>
+  <si>
+    <t>Vous allez maintenant effectuer un bloc d'essais,&lt;br&gt;au cours desquels nous mesurerons vos données.&lt;br&gt;&lt;b&gt;Chaque essai compte.&lt;/b&gt;</t>
+  </si>
+  <si>
+    <t>Vous allez maintenant effectuer &lt;b&gt;4 blocs&lt;/b&gt; d'essais,&lt;br&gt;au cours desquels nous mesurerons vos données.&lt;br&gt;&lt;b&gt;Chaque essai compte.&lt;/b&gt;&lt;br&gt;&lt;br&gt;Entre les blocs, vous pouvez faire une pause.&lt;br&gt;&lt;br&gt;Le premier bloc commence lorsque vous appuyez sur la touche ESPACE.</t>
+  </si>
+  <si>
+    <t>Le sigue ahora el segundo bloque.&lt;br&gt;&lt;br&gt;Recordatorio: responda de la forma más &lt;b&gt;rápida y correcta&lt;/b&gt; posible.</t>
+  </si>
+  <si>
+    <t>Le deuxième bloc suit maintenant.&lt;br&gt;&lt;br&gt;Rappel : répondez aussi &lt;b&gt;rapidement et correctement&lt;/b&gt; que possible.</t>
+  </si>
+  <si>
+    <t>Le sigue ahora el tercer bloque.&lt;br&gt;&lt;br&gt;Recordatorio: responda de la forma más &lt;b&gt;rápida y correcta&lt;/b&gt; posible.</t>
+  </si>
+  <si>
+    <t>Le troisième bloc suit maintenant.&lt;br&gt;&lt;br&gt;Rappel : répondez aussi &lt;b&gt;rapidement et correctement&lt;/b&gt; que possible.</t>
+  </si>
+  <si>
+    <t>Le sigue ahora el último bloque.&lt;br&gt;&lt;br&gt;Recordatorio: responda de la forma más &lt;b&gt;rápida y correcta&lt;/b&gt; posible.</t>
+  </si>
+  <si>
+    <t>Le dernier bloc suit maintenant.&lt;br&gt;&lt;br&gt;Rappel : répondez aussi &lt;b&gt;rapidement et correctement&lt;/b&gt; que possible.</t>
   </si>
 </sst>
 </file>
@@ -166,9 +239,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -206,7 +279,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -312,7 +385,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -454,7 +527,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -462,16 +535,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D84571D-E185-45F8-BE88-DC2A982E2C1F}">
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.73046875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:L5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="40.625" defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.73046875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="184.86328125" style="1" customWidth="1"/>
-    <col min="3" max="6" width="40.73046875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="40.73046875" customWidth="1"/>
+    <col min="1" max="16384" width="40.625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
@@ -490,8 +560,26 @@
       <c r="F1" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" ht="85.5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" ht="99.85" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
@@ -510,8 +598,26 @@
       <c r="F2" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="G2" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>25</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" ht="42.8" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>18</v>
       </c>
@@ -524,8 +630,20 @@
       <c r="F3" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
-    <row r="4" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" ht="42.8" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>19</v>
       </c>
@@ -538,8 +656,20 @@
       <c r="F4" s="1" t="s">
         <v>6</v>
       </c>
+      <c r="H4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="5" spans="1:6" ht="42.75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" ht="42.8" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>20</v>
       </c>
@@ -551,6 +681,18 @@
       </c>
       <c r="F5" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>